<commit_message>
docs(tutorials): FEM-3 — the wall is driven into the base: one run with Tip = fixed, the pinned wall run and 'Fixing the toe' removed; engine table narrowed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_johnson_rapid.xlsx
+++ b/docs/tutorials/files/xslope_johnson_rapid.xlsx
@@ -5126,7 +5126,7 @@
         </is>
       </c>
       <c r="F3" s="35">
-        <v>100.0</v>
+        <v>110.0</v>
       </c>
       <c r="H3" s="34" t="inlineStr">
         <is>
@@ -5197,8 +5197,12 @@
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="B5" s="3">
+        <v>380.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>180.0</v>
+      </c>
       <c r="E5" s="3">
         <v>0.0</v>
       </c>
@@ -5225,8 +5229,12 @@
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="3">
+        <v>550.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>100.0</v>
+      </c>
       <c r="E6" s="3">
         <v>200.0</v>
       </c>
@@ -5249,8 +5257,12 @@
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="E7" s="3">
+        <v>220.0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>110.0</v>
+      </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="K7" s="3"/>
@@ -5587,7 +5599,7 @@
         <v>50.0</v>
       </c>
       <c r="C5" s="3">
-        <v>100.0</v>
+        <v>110.0</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -11402,7 +11414,7 @@
         <v>0.0</v>
       </c>
       <c r="E5" s="3">
-        <v>100.0</v>
+        <v>110.0</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>18</v>
@@ -11419,10 +11431,10 @@
         <v>160.0</v>
       </c>
       <c r="D6" s="3">
-        <v>200.0</v>
+        <v>220.0</v>
       </c>
       <c r="E6" s="3">
-        <v>100.0</v>
+        <v>110.0</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>192</v>
@@ -11442,7 +11454,7 @@
         <v>360.0</v>
       </c>
       <c r="E7" s="3">
-        <v>150.0</v>
+        <v>107.0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -11456,7 +11468,7 @@
         <v>410.0</v>
       </c>
       <c r="E8" s="3">
-        <v>120.0</v>
+        <v>103.0</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
docs(tutorials): COMBO-2 — seepage figures are the result tabs as Studio draws them; readers clear the piezometric lines at Part 2 and Set 2 at Part 3; completed workbook ships without the lines
Also carries the lem13_sweeps producer group (page placeholders still pending).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_johnson_rapid.xlsx
+++ b/docs/tutorials/files/xslope_johnson_rapid.xlsx
@@ -11404,18 +11404,10 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B5" s="3">
-        <v>160.0</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>110.0</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
       <c r="G5" s="1" t="s">
         <v>18</v>
       </c>
@@ -11424,18 +11416,10 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>360.0</v>
-      </c>
-      <c r="B6" s="3">
-        <v>160.0</v>
-      </c>
-      <c r="D6" s="3">
-        <v>220.0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>110.0</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
         <v>192</v>
       </c>
@@ -11444,56 +11428,28 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>410.0</v>
-      </c>
-      <c r="B7" s="3">
-        <v>120.0</v>
-      </c>
-      <c r="D7" s="3">
-        <v>360.0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>107.0</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>550.0</v>
-      </c>
-      <c r="B8" s="3">
-        <v>100.0</v>
-      </c>
-      <c r="D8" s="3">
-        <v>410.0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>103.0</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>750.0</v>
-      </c>
-      <c r="B9" s="3">
-        <v>100.0</v>
-      </c>
-      <c r="D9" s="3">
-        <v>550.0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
-      <c r="D10" s="3">
-        <v>750.0</v>
-      </c>
-      <c r="E10" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>

</xml_diff>